<commit_message>
ETL: corrige cache Rentabilidade, formula ganho liquido, NFD sem transportadora
</commit_message>
<xml_diff>
--- a/data/Base_Intelipost_Resumo.xlsx
+++ b/data/Base_Intelipost_Resumo.xlsx
@@ -441,22 +441,22 @@
         <v>0</v>
       </c>
       <c r="D2">
-        <v>252343652.9299999</v>
+        <v>260613956.04</v>
       </c>
       <c r="E2">
-        <v>16776782.31</v>
+        <v>17185422.44</v>
       </c>
       <c r="F2">
-        <v>16413</v>
+        <v>16482</v>
       </c>
       <c r="G2">
-        <v>627</v>
+        <v>633</v>
       </c>
       <c r="H2">
-        <v>47662</v>
+        <v>48829</v>
       </c>
       <c r="I2">
-        <v>13579</v>
+        <v>13617</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao Monitor (upload web)
</commit_message>
<xml_diff>
--- a/data/Base_Intelipost_Resumo.xlsx
+++ b/data/Base_Intelipost_Resumo.xlsx
@@ -432,10 +432,10 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2">
-        <v>1144654</v>
+        <v>1188159</v>
       </c>
       <c r="B2">
-        <v>254378835.0100001</v>
+        <v>263686820.63</v>
       </c>
       <c r="C2">
         <v>0</v>

</xml_diff>

<commit_message>
Trade-off: corrige meses futuros, JET sem despacho, vendas por transportadora e debug TSP
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Base_Intelipost_Resumo.xlsx
+++ b/data/Base_Intelipost_Resumo.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>TotalPedidos</t>
   </si>
@@ -41,12 +41,24 @@
   </si>
   <si>
     <t>NFDTranspPRWFallback</t>
+  </si>
+  <si>
+    <t>UltimaDataVenda</t>
+  </si>
+  <si>
+    <t>UltimaDataDespacho</t>
+  </si>
+  <si>
+    <t>AtualizadoEm</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -99,11 +111,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -398,10 +411,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -429,8 +442,17 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:12">
       <c r="A2">
         <v>1301127</v>
       </c>
@@ -457,6 +479,15 @@
       </c>
       <c r="I2">
         <v>14228</v>
+      </c>
+      <c r="J2" s="2">
+        <v>46285</v>
+      </c>
+      <c r="K2" s="2">
+        <v>46308.08803688658</v>
+      </c>
+      <c r="L2" s="2">
+        <v>46308.41423370193</v>
       </c>
     </row>
   </sheetData>

</xml_diff>